<commit_message>
fixed score screen sizing, and score screen registry logic for discontinued experiment sessions
</commit_message>
<xml_diff>
--- a/blocks_final.xlsx
+++ b/blocks_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Backups\All Files\Genel\Is\2022\Upwork\LabX\studies\materials\drivingSimulator\repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CFA99FD-02B2-461B-ADB3-AF5C29BE1C05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45D8152-8988-416C-83CF-3C198E6C3187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="25875" windowHeight="14175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="36">
   <si>
     <t>current_font</t>
   </si>
@@ -130,6 +130,18 @@
   </si>
   <si>
     <t>./instructions_pilot/clutterlex_training.png</t>
+  </si>
+  <si>
+    <t>scoreRegistry</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t>lexical_only</t>
+  </si>
+  <si>
+    <t>driving_lexical</t>
   </si>
 </sst>
 </file>
@@ -447,7 +459,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultColWidth="12.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.7109375" customWidth="1"/>
@@ -455,7 +467,7 @@
     <col min="8" max="8" width="64.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -492,8 +504,11 @@
       <c r="L1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -530,8 +545,11 @@
       <c r="L2" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -568,8 +586,11 @@
       <c r="L3" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -606,8 +627,11 @@
       <c r="L4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -644,8 +668,11 @@
       <c r="L5" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -682,8 +709,11 @@
       <c r="L6" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -720,8 +750,11 @@
       <c r="L7" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -758,8 +791,11 @@
       <c r="L8" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -796,8 +832,11 @@
       <c r="L9" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -833,6 +872,9 @@
       </c>
       <c r="L10" t="b">
         <v>1</v>
+      </c>
+      <c r="M10" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added whitespace after first instructions
</commit_message>
<xml_diff>
--- a/blocks_final.xlsx
+++ b/blocks_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Backups\All Files\Genel\Is\2022\Upwork\LabX\studies\materials\drivingSimulator\repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45D8152-8988-416C-83CF-3C198E6C3187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{469829D3-9A03-4B06-81D3-804CFF4021EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="25875" windowHeight="14175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>